<commit_message>
feat: synchronize competition deliverables with official cloud links and presentation deck
</commit_message>
<xml_diff>
--- a/2_Excel_Nextute_Case_B_Financial_Model.xlsx
+++ b/2_Excel_Nextute_Case_B_Financial_Model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\AppData\Roaming\Microsoft\Windows\Network Shortcuts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68A26F8B-6F0F-4D1C-8F09-7C8235D93CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{39F5D549-BC41-4096-8A0B-4C155E99DABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
feat: sync 2_Excel_Nextute_Case_B_Financial_Model.xlsx with latest live OneDrive version
</commit_message>
<xml_diff>
--- a/2_Excel_Nextute_Case_B_Financial_Model.xlsx
+++ b/2_Excel_Nextute_Case_B_Financial_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\AppData\Roaming\Microsoft\Windows\Network Shortcuts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39F5D549-BC41-4096-8A0B-4C155E99DABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{18AEB019-3309-4B0C-8428-500283D29251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9D82A5F-D7E1-47D2-A1C9-C85582065934}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7875" firstSheet="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions &amp; Drivers" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="192">
+  <si>
+    <t>IntelliPrivart</t>
+  </si>
   <si>
     <t>NEXTUTE EDTECH - CASE B: THE DATA MOAT</t>
   </si>
@@ -132,6 +135,9 @@
     <t>Tier 2: Additional Student Variable Fee</t>
   </si>
   <si>
+    <t>INR / Student/Month</t>
+  </si>
+  <si>
     <t>Per student above 300</t>
   </si>
   <si>
@@ -144,7 +150,7 @@
     <t>Tier 3: Enterprise Rate (&gt;600 Students)</t>
   </si>
   <si>
-    <t>INR / Student / Mo</t>
+    <t>INR / Student / Month</t>
   </si>
   <si>
     <t>Custom volume pricing</t>
@@ -363,7 +369,7 @@
     <t>Benchmark / Comment</t>
   </si>
   <si>
-    <t>Monthly Revenue per Institute (ARPA)</t>
+    <t>Monthly Revenue per Institute (MRPA)</t>
   </si>
   <si>
     <t>Tier 2 hybrid plan for 400 students</t>
@@ -623,7 +629,7 @@
     <numFmt numFmtId="167" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -698,6 +704,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF1F497D"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -792,7 +805,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -809,21 +822,30 @@
     <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -842,15 +864,44 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1153,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:E35"/>
+  <dimension ref="B1:G35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1163,412 +1214,453 @@
     <col min="5" max="5" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="19.5">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="2:7" ht="18.75">
+      <c r="B1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-    </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="2" t="s">
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="2:7" ht="19.5">
+      <c r="B2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-    </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="25" t="s">
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7">
+      <c r="B3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-    </row>
-    <row r="7" spans="2:5">
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="19"/>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+    </row>
+    <row r="7" spans="2:7">
       <c r="B7" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" s="4">
         <v>400</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5">
+        <v>6</v>
+      </c>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+    </row>
+    <row r="8" spans="2:7">
       <c r="B8" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="6">
         <v>60000</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5">
+        <v>9</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+    </row>
+    <row r="9" spans="2:7">
       <c r="B9" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="4">
         <v>10</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5">
+        <v>12</v>
+      </c>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+    </row>
+    <row r="10" spans="2:7">
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="6">
         <f>C8/C9</f>
         <v>6000</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5">
+        <v>15</v>
+      </c>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+    </row>
+    <row r="11" spans="2:7">
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="7">
         <v>0.12</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5">
+        <v>18</v>
+      </c>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+    </row>
+    <row r="12" spans="2:7">
       <c r="B12" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" s="4">
         <v>4</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5">
+        <v>21</v>
+      </c>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+    </row>
+    <row r="13" spans="2:7">
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="6">
         <f>C10*(C9-C12)</f>
         <v>36000</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5">
-      <c r="B14" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-    </row>
-    <row r="15" spans="2:5">
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-    </row>
-    <row r="16" spans="2:5">
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7">
       <c r="B16" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C16" s="6">
         <v>5999</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>26</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" s="6">
         <v>9999</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" s="6">
         <v>30</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C19" s="6">
         <f>C17+(400-300)*C18</f>
         <v>12999</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C20" s="6">
         <v>28</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
+      <c r="B21" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
     </row>
     <row r="22" spans="2:5">
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C23" s="8">
         <v>2</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="2:5">
       <c r="B24" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C24" s="8">
         <v>2.5</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C25" s="8">
         <v>4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="2:5">
       <c r="B26" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C26" s="8">
         <v>0.5</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C27" s="8">
         <f>SUM(C23:C26)</f>
         <v>9</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="2:5">
-      <c r="B28" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
+      <c r="B28" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
     </row>
     <row r="29" spans="2:5">
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C30" s="6">
         <v>24000</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C31" s="6">
         <v>6000</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="2:5">
       <c r="B32" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C32" s="6">
         <f>C30+C31</f>
         <v>30000</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C33" s="4">
         <v>4</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="2:5">
       <c r="B34" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C34" s="7">
         <v>0.12</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C35" s="7">
         <f>1-(1-C34)^(1/12)</f>
         <v>1.0596241035318976E-2</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
     <mergeCell ref="B5:E6"/>
     <mergeCell ref="B14:E15"/>
     <mergeCell ref="B21:E22"/>
     <mergeCell ref="B28:E29"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1589,255 +1681,255 @@
   <sheetData>
     <row r="2" spans="2:5" ht="19.5">
       <c r="B2" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+        <v>66</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
+        <v>67</v>
+      </c>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
     </row>
     <row r="5" spans="2:5">
-      <c r="B5" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="23" t="s">
+      <c r="B5" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="C5" s="17" t="s">
         <v>69</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C6" s="4">
         <f>'Assumptions &amp; Drivers'!C7</f>
         <v>400</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6">
         <f>'Assumptions &amp; Drivers'!C8</f>
         <v>60000</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C8" s="6">
         <f>C6*C7</f>
         <v>24000000</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C9" s="7">
         <f>'Assumptions &amp; Drivers'!C11</f>
         <v>0.12</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="4">
         <f>C6*C9</f>
         <v>48</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C11" s="6">
         <f>'Assumptions &amp; Drivers'!C13</f>
         <v>36000</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C12" s="6">
         <f>C10*C11</f>
         <v>1728000</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="2:5">
-      <c r="B13" s="31" t="s">
-        <v>85</v>
-      </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
+      <c r="B13" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
     </row>
     <row r="14" spans="2:5">
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
     </row>
     <row r="15" spans="2:5">
-      <c r="B15" s="22" t="s">
-        <v>86</v>
+      <c r="B15" s="16" t="s">
+        <v>88</v>
       </c>
       <c r="C15" s="7">
         <v>0.15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C16" s="4">
         <f>ROUND(C10*C15, 0)</f>
         <v>7</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C17" s="6">
         <f>C16*C11</f>
         <v>252000</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C18" s="6">
         <f>'Assumptions &amp; Drivers'!C19*'Assumptions &amp; Drivers'!C9</f>
         <v>129990</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C19" s="6">
         <f>C17-C18</f>
         <v>122010</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C20" s="11">
         <f>C17/C18</f>
         <v>1.938610662358643</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="22" t="s">
-        <v>100</v>
+      <c r="B21" s="16" t="s">
+        <v>102</v>
       </c>
       <c r="C21" s="12">
         <f>C18/C11</f>
         <v>3.6108333333333333</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1855,314 +1947,314 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="64" customWidth="1"/>
+    <col min="3" max="3" width="34.140625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="19.5">
-      <c r="B2" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="B2" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
     </row>
     <row r="3" spans="2:5">
-      <c r="B3" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
+      <c r="B3" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C6" s="6">
         <f>'Assumptions &amp; Drivers'!C19</f>
         <v>12999</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C7" s="6">
         <f>'Assumptions &amp; Drivers'!C27*'Assumptions &amp; Drivers'!C7</f>
         <v>3600</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C8" s="6">
         <v>1800</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C9" s="6">
         <f>C7+C8</f>
         <v>5400</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C10" s="6">
         <f>C6-C9</f>
         <v>7599</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C11" s="7">
         <f>C10/C6</f>
         <v>0.58458342949457653</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="2:5">
-      <c r="B12" s="33"/>
+      <c r="B12" s="34" t="s">
+        <v>121</v>
+      </c>
       <c r="C12" s="34"/>
       <c r="D12" s="34"/>
       <c r="E12" s="34"/>
     </row>
     <row r="13" spans="2:5">
-      <c r="B13" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C14" s="6">
         <f>'Assumptions &amp; Drivers'!C30</f>
         <v>24000</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C15" s="6">
         <f>'Assumptions &amp; Drivers'!C31</f>
         <v>6000</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C16" s="6">
         <f>C14+C15</f>
         <v>30000</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C17" s="13">
         <f>C16/C10</f>
         <v>3.9478878799842083</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="2:5">
-      <c r="B18" s="33"/>
+      <c r="B18" s="34" t="s">
+        <v>130</v>
+      </c>
       <c r="C18" s="34"/>
       <c r="D18" s="34"/>
       <c r="E18" s="34"/>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="33" t="s">
-        <v>128</v>
-      </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C20" s="7">
         <f>'Assumptions &amp; Drivers'!C34</f>
         <v>0.12</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C21" s="13">
         <f>1/C20</f>
         <v>8.3333333333333339</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C22" s="13">
         <f>C21*12</f>
         <v>100</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C23" s="13">
         <f>C21*'Assumptions &amp; Drivers'!C9</f>
         <v>83.333333333333343</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="2:5">
       <c r="B24" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C24" s="6">
         <f>C23*C10</f>
         <v>633250.00000000012</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C25" s="11">
         <f>C24/C16</f>
         <v>21.108333333333338</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B12:E13"/>
+    <mergeCell ref="B18:E19"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2180,110 +2272,112 @@
   <sheetData>
     <row r="2" spans="2:9" ht="19.5">
       <c r="B2" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+        <v>144</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="2:9">
       <c r="B3" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
+        <v>145</v>
+      </c>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
     </row>
     <row r="5" spans="2:9">
       <c r="B5" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="2:9">
       <c r="B6" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="C6" s="14">
+        <v>154</v>
+      </c>
+      <c r="C6" s="38">
         <v>10</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="38">
         <v>20</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="38">
         <v>35</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="38">
         <v>50</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="38">
         <f>F6</f>
         <v>50</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="38">
         <v>180</v>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="38">
         <v>520</v>
       </c>
     </row>
     <row r="7" spans="2:9">
       <c r="B7" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C7" s="14">
+        <v>155</v>
+      </c>
+      <c r="C7" s="38">
         <v>4000</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="38">
         <v>8000</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="38">
         <v>14000</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="38">
         <v>20000</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="38">
         <f>F7</f>
         <v>20000</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="38">
         <v>72000</v>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="38">
         <v>208000</v>
       </c>
     </row>
     <row r="8" spans="2:9">
-      <c r="B8" s="33"/>
+      <c r="B8" s="34" t="s">
+        <v>156</v>
+      </c>
       <c r="C8" s="34"/>
       <c r="D8" s="34"/>
       <c r="E8" s="34"/>
@@ -2293,106 +2387,106 @@
       <c r="I8" s="34"/>
     </row>
     <row r="9" spans="2:9">
-      <c r="B9" s="33" t="s">
-        <v>154</v>
-      </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
     </row>
     <row r="10" spans="2:9">
       <c r="B10" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C10" s="15">
+        <v>157</v>
+      </c>
+      <c r="C10" s="39">
         <v>3.9</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="39">
         <v>7.8</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="39">
         <v>13.65</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="39">
         <v>19.5</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="39">
         <f>SUM(C10:F10)</f>
         <v>44.85</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="39">
         <v>187.2</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="39">
         <v>594.88</v>
       </c>
     </row>
     <row r="11" spans="2:9">
       <c r="B11" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C11" s="15">
+        <v>158</v>
+      </c>
+      <c r="C11" s="39">
         <v>0.6</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="39">
         <v>1.2</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="39">
         <v>2.1</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="39">
         <v>3</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="39">
         <f>SUM(C11:F11)</f>
         <v>6.9</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="39">
         <v>32.4</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="39">
         <v>112.32</v>
       </c>
     </row>
     <row r="12" spans="2:9">
       <c r="B12" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="C12" s="8">
+        <v>159</v>
+      </c>
+      <c r="C12" s="40">
         <f>C10+C11</f>
         <v>4.5</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="40">
         <f>D10+D11</f>
         <v>9</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="40">
         <f>E10+E11</f>
         <v>15.75</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="40">
         <f>F10+F11</f>
         <v>22.5</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="40">
         <f>SUM(G10:G11)</f>
         <v>51.75</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="40">
         <f>H10+H11</f>
         <v>219.6</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="40">
         <f>I10+I11</f>
         <v>707.2</v>
       </c>
     </row>
     <row r="13" spans="2:9">
-      <c r="B13" s="33"/>
+      <c r="B13" s="34" t="s">
+        <v>160</v>
+      </c>
       <c r="C13" s="34"/>
       <c r="D13" s="34"/>
       <c r="E13" s="34"/>
@@ -2402,226 +2496,226 @@
       <c r="I13" s="34"/>
     </row>
     <row r="14" spans="2:9">
-      <c r="B14" s="33" t="s">
-        <v>158</v>
-      </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
     </row>
     <row r="15" spans="2:9">
       <c r="B15" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C15" s="15">
+        <v>161</v>
+      </c>
+      <c r="C15" s="39">
         <v>0.24</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="39">
         <v>0.48</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="39">
         <v>0.84</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="39">
         <v>1.2</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="39">
         <f>SUM(C15:F15)</f>
         <v>2.76</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="39">
         <v>12.96</v>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="39">
         <v>41.6</v>
       </c>
     </row>
     <row r="16" spans="2:9">
       <c r="B16" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C16" s="15">
+        <v>162</v>
+      </c>
+      <c r="C16" s="39">
         <v>0.3</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="39">
         <v>0.6</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="39">
         <v>1.05</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="39">
         <v>1.5</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="39">
         <f>SUM(C16:F16)</f>
         <v>3.45</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="39">
         <v>16.2</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="39">
         <v>52</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="C17" s="15">
+        <v>163</v>
+      </c>
+      <c r="C17" s="39">
         <v>0.48</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="39">
         <v>0.96</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="39">
         <v>1.68</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="39">
         <v>2.4</v>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="39">
         <f>SUM(C17:F17)</f>
         <v>5.52</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="39">
         <v>25.92</v>
       </c>
-      <c r="I17" s="15">
+      <c r="I17" s="39">
         <v>83.2</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="C18" s="15">
+        <v>164</v>
+      </c>
+      <c r="C18" s="39">
         <v>0.54</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="39">
         <v>1.08</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="39">
         <v>1.89</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="39">
         <v>2.7</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="39">
         <f>SUM(C18:F18)</f>
         <v>6.21</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="39">
         <v>23.33</v>
       </c>
-      <c r="I18" s="15">
+      <c r="I18" s="39">
         <v>67.39</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="C19" s="8">
+        <v>165</v>
+      </c>
+      <c r="C19" s="40">
         <f t="shared" ref="C19:I19" si="0">SUM(C15:C18)</f>
         <v>1.56</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="40">
         <f t="shared" si="0"/>
         <v>3.12</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="40">
         <f t="shared" si="0"/>
         <v>5.46</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="40">
         <f t="shared" si="0"/>
         <v>7.8</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="40">
         <f t="shared" si="0"/>
         <v>17.940000000000001</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="40">
         <f t="shared" si="0"/>
         <v>78.41</v>
       </c>
-      <c r="I19" s="8">
+      <c r="I19" s="40">
         <f t="shared" si="0"/>
         <v>244.19</v>
       </c>
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="C20" s="8">
+        <v>166</v>
+      </c>
+      <c r="C20" s="40">
         <f t="shared" ref="C20:I20" si="1">C12-C19</f>
         <v>2.94</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="40">
         <f t="shared" si="1"/>
         <v>5.88</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="40">
         <f t="shared" si="1"/>
         <v>10.29</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="40">
         <f t="shared" si="1"/>
         <v>14.7</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="40">
         <f t="shared" si="1"/>
         <v>33.81</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="40">
         <f t="shared" si="1"/>
         <v>141.19</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="40">
         <f t="shared" si="1"/>
         <v>463.01000000000005</v>
       </c>
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C21" s="16">
+        <v>119</v>
+      </c>
+      <c r="C21" s="41">
         <f t="shared" ref="C21:I21" si="2">C20/C12</f>
         <v>0.65333333333333332</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="41">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="41">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="41">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="41">
         <f t="shared" si="2"/>
         <v>0.65333333333333343</v>
       </c>
-      <c r="H21" s="16">
+      <c r="H21" s="41">
         <f t="shared" si="2"/>
         <v>0.64294171220400731</v>
       </c>
-      <c r="I21" s="16">
+      <c r="I21" s="41">
         <f t="shared" si="2"/>
         <v>0.65470871040723988</v>
       </c>
     </row>
     <row r="22" spans="2:9">
-      <c r="B22" s="33"/>
+      <c r="B22" s="34" t="s">
+        <v>167</v>
+      </c>
       <c r="C22" s="34"/>
       <c r="D22" s="34"/>
       <c r="E22" s="34"/>
@@ -2631,216 +2725,211 @@
       <c r="I22" s="34"/>
     </row>
     <row r="23" spans="2:9">
-      <c r="B23" s="33" t="s">
-        <v>165</v>
-      </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C24" s="15">
+        <v>168</v>
+      </c>
+      <c r="C24" s="39">
         <v>3</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="39">
         <v>3</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="39">
         <v>4.5</v>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="39">
         <v>4.5</v>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="39">
         <f>SUM(C24:F24)</f>
         <v>15</v>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="39">
         <v>39</v>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="39">
         <v>102</v>
       </c>
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C25" s="15">
+        <v>169</v>
+      </c>
+      <c r="C25" s="39">
         <v>6</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="39">
         <v>6</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="39">
         <v>7.5</v>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="39">
         <v>7.5</v>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="39">
         <f>SUM(C25:F25)</f>
         <v>27</v>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="39">
         <v>42</v>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="39">
         <v>78</v>
       </c>
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C26" s="15">
+        <v>170</v>
+      </c>
+      <c r="C26" s="39">
         <v>1.5</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="39">
         <v>1.5</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="39">
         <v>2</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="39">
         <v>2</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="39">
         <f>SUM(C26:F26)</f>
         <v>7</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="39">
         <v>12</v>
       </c>
-      <c r="I26" s="15">
+      <c r="I26" s="39">
         <v>24</v>
       </c>
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="C27" s="8">
+        <v>171</v>
+      </c>
+      <c r="C27" s="40">
         <f t="shared" ref="C27:I27" si="3">SUM(C24:C26)</f>
         <v>10.5</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27" s="40">
         <f t="shared" si="3"/>
         <v>10.5</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="40">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="40">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="40">
         <f t="shared" si="3"/>
         <v>49</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="40">
         <f t="shared" si="3"/>
         <v>93</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="40">
         <f t="shared" si="3"/>
         <v>204</v>
       </c>
     </row>
     <row r="28" spans="2:9">
-      <c r="B28" s="33"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
     </row>
     <row r="29" spans="2:9">
       <c r="B29" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="C29" s="17">
+        <v>172</v>
+      </c>
+      <c r="C29" s="42">
         <f t="shared" ref="C29:I29" si="4">C20-C27</f>
         <v>-7.5600000000000005</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="42">
         <f t="shared" si="4"/>
         <v>-4.62</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="42">
         <f t="shared" si="4"/>
         <v>-3.7100000000000009</v>
       </c>
-      <c r="F29" s="17">
+      <c r="F29" s="42">
         <f t="shared" si="4"/>
         <v>0.69999999999999929</v>
       </c>
-      <c r="G29" s="17">
+      <c r="G29" s="42">
         <f t="shared" si="4"/>
         <v>-15.189999999999998</v>
       </c>
-      <c r="H29" s="17">
+      <c r="H29" s="42">
         <f t="shared" si="4"/>
         <v>48.19</v>
       </c>
-      <c r="I29" s="17">
+      <c r="I29" s="42">
         <f t="shared" si="4"/>
         <v>259.01000000000005</v>
       </c>
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C30" s="16">
+        <v>173</v>
+      </c>
+      <c r="C30" s="41">
         <f t="shared" ref="C30:I30" si="5">C29/C12</f>
         <v>-1.6800000000000002</v>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="41">
         <f t="shared" si="5"/>
         <v>-0.51333333333333331</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="41">
         <f t="shared" si="5"/>
         <v>-0.2355555555555556</v>
       </c>
-      <c r="F30" s="16">
+      <c r="F30" s="41">
         <f t="shared" si="5"/>
         <v>3.1111111111111079E-2</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="41">
         <f t="shared" si="5"/>
         <v>-0.29352657004830912</v>
       </c>
-      <c r="H30" s="16">
+      <c r="H30" s="41">
         <f t="shared" si="5"/>
         <v>0.21944444444444444</v>
       </c>
-      <c r="I30" s="16">
+      <c r="I30" s="41">
         <f t="shared" si="5"/>
         <v>0.36624717194570139</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B13:I13"/>
+  <mergeCells count="4">
     <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B22:I22"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B8:I9"/>
+    <mergeCell ref="B13:I14"/>
+    <mergeCell ref="B22:I23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2852,68 +2941,72 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="8" width="52" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="19.5">
       <c r="B2" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+        <v>174</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
+        <v>175</v>
+      </c>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
     </row>
     <row r="5" spans="2:8">
-      <c r="B5" s="35" t="s">
-        <v>174</v>
-      </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
+      <c r="B5" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
     </row>
     <row r="6" spans="2:8">
-      <c r="B6" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="19">
+      <c r="B6" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="15">
         <v>40000</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="15">
         <v>50000</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="15">
         <v>60000</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="15">
         <v>75000</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="15">
         <v>90000</v>
       </c>
     </row>
     <row r="7" spans="2:8">
-      <c r="B7" s="18" t="s">
-        <v>176</v>
+      <c r="B7" s="14" t="s">
+        <v>178</v>
       </c>
       <c r="C7" s="20">
         <v>0.05</v>
@@ -2940,8 +3033,8 @@
       </c>
     </row>
     <row r="8" spans="2:8">
-      <c r="B8" s="18" t="s">
-        <v>177</v>
+      <c r="B8" s="14" t="s">
+        <v>179</v>
       </c>
       <c r="C8" s="20">
         <v>0.1</v>
@@ -2968,8 +3061,8 @@
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="18" t="s">
-        <v>178</v>
+      <c r="B9" s="14" t="s">
+        <v>180</v>
       </c>
       <c r="C9" s="20">
         <v>0.15</v>
@@ -2996,8 +3089,8 @@
       </c>
     </row>
     <row r="10" spans="2:8">
-      <c r="B10" s="18" t="s">
-        <v>179</v>
+      <c r="B10" s="14" t="s">
+        <v>181</v>
       </c>
       <c r="C10" s="20">
         <v>0.2</v>
@@ -3024,8 +3117,8 @@
       </c>
     </row>
     <row r="11" spans="2:8">
-      <c r="B11" s="18" t="s">
-        <v>180</v>
+      <c r="B11" s="14" t="s">
+        <v>182</v>
       </c>
       <c r="C11" s="20">
         <v>0.25</v>
@@ -3053,50 +3146,50 @@
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
+        <v>183</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="35" t="s">
-        <v>182</v>
-      </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
+      <c r="B16" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="19">
+      <c r="B17" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="15">
         <v>20000</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="15">
         <v>25000</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="15">
         <v>30000</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="15">
         <v>35000</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="15">
         <v>40000</v>
       </c>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="18" t="s">
-        <v>184</v>
+      <c r="B18" s="14" t="s">
+        <v>186</v>
       </c>
       <c r="C18" s="20">
         <v>0.08</v>
@@ -3123,8 +3216,8 @@
       </c>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="18" t="s">
-        <v>185</v>
+      <c r="B19" s="14" t="s">
+        <v>187</v>
       </c>
       <c r="C19" s="20">
         <v>0.1</v>
@@ -3151,8 +3244,8 @@
       </c>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="18" t="s">
-        <v>186</v>
+      <c r="B20" s="14" t="s">
+        <v>188</v>
       </c>
       <c r="C20" s="20">
         <v>0.12</v>
@@ -3179,8 +3272,8 @@
       </c>
     </row>
     <row r="21" spans="2:8">
-      <c r="B21" s="18" t="s">
-        <v>187</v>
+      <c r="B21" s="14" t="s">
+        <v>189</v>
       </c>
       <c r="C21" s="20">
         <v>0.15</v>
@@ -3207,8 +3300,8 @@
       </c>
     </row>
     <row r="22" spans="2:8">
-      <c r="B22" s="18" t="s">
-        <v>188</v>
+      <c r="B22" s="14" t="s">
+        <v>190</v>
       </c>
       <c r="C22" s="20">
         <v>0.2</v>
@@ -3236,14 +3329,14 @@
     </row>
     <row r="24" spans="2:8">
       <c r="B24" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
+        <v>191</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
fix(financial-model): update Excel workbooks and public assets with revised financial model and unit economics
</commit_message>
<xml_diff>
--- a/2_Excel_Nextute_Case_B_Financial_Model.xlsx
+++ b/2_Excel_Nextute_Case_B_Financial_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\AppData\Roaming\Microsoft\Windows\Network Shortcuts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{18AEB019-3309-4B0C-8428-500283D29251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9D82A5F-D7E1-47D2-A1C9-C85582065934}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AABBE1C-C45C-4243-A42F-A0D8E443E3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7875" firstSheet="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions &amp; Drivers" sheetId="1" r:id="rId1"/>
@@ -840,11 +840,20 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -863,6 +872,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -884,23 +896,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1215,50 +1215,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18.75">
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
     </row>
     <row r="2" spans="2:7" ht="19.5">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
       <c r="F2" s="18"/>
       <c r="G2" s="18"/>
     </row>
     <row r="3" spans="2:7">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
       <c r="F3" s="18"/>
       <c r="G3" s="18"/>
     </row>
     <row r="5" spans="2:7">
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
       <c r="F5" s="18"/>
       <c r="G5" s="19"/>
     </row>
     <row r="6" spans="2:7">
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
       <c r="F6" s="18"/>
       <c r="G6" s="18"/>
     </row>
@@ -1377,20 +1377,20 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
       <c r="F14" s="18"/>
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="2:7">
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
       <c r="F15" s="18"/>
       <c r="G15" s="18"/>
     </row>
@@ -1468,18 +1468,18 @@
       </c>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
     </row>
     <row r="22" spans="2:5">
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
     </row>
     <row r="23" spans="2:5">
       <c r="B23" s="3" t="s">
@@ -1553,18 +1553,18 @@
       </c>
     </row>
     <row r="28" spans="2:5">
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
     </row>
     <row r="29" spans="2:5">
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
+      <c r="B29" s="32"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="3" t="s">
@@ -1815,18 +1815,18 @@
       </c>
     </row>
     <row r="13" spans="2:5">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="36" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
     </row>
     <row r="14" spans="2:5">
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="16" t="s">
@@ -1953,20 +1953,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="19.5">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="3" spans="2:5">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="9" t="s">
@@ -2072,18 +2072,18 @@
       </c>
     </row>
     <row r="12" spans="2:5">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
     </row>
     <row r="13" spans="2:5">
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="3" t="s">
@@ -2146,18 +2146,18 @@
       </c>
     </row>
     <row r="18" spans="2:5">
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="2:5">
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="3" t="s">
@@ -2324,26 +2324,26 @@
       <c r="B6" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="22">
         <v>10</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="22">
         <v>20</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="22">
         <v>35</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="22">
         <v>50</v>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="22">
         <f>F6</f>
         <v>50</v>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="22">
         <v>180</v>
       </c>
-      <c r="I6" s="38">
+      <c r="I6" s="22">
         <v>520</v>
       </c>
     </row>
@@ -2351,75 +2351,75 @@
       <c r="B7" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="22">
         <v>4000</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="22">
         <v>8000</v>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="22">
         <v>14000</v>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="22">
         <v>20000</v>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="22">
         <f>F7</f>
         <v>20000</v>
       </c>
-      <c r="H7" s="38">
+      <c r="H7" s="22">
         <v>72000</v>
       </c>
-      <c r="I7" s="38">
+      <c r="I7" s="22">
         <v>208000</v>
       </c>
     </row>
     <row r="8" spans="2:9">
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
     </row>
     <row r="9" spans="2:9">
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="2:9">
       <c r="B10" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C10" s="39">
+      <c r="C10" s="23">
         <v>3.9</v>
       </c>
-      <c r="D10" s="39">
+      <c r="D10" s="23">
         <v>7.8</v>
       </c>
-      <c r="E10" s="39">
+      <c r="E10" s="23">
         <v>13.65</v>
       </c>
-      <c r="F10" s="39">
+      <c r="F10" s="23">
         <v>19.5</v>
       </c>
-      <c r="G10" s="39">
+      <c r="G10" s="23">
         <f>SUM(C10:F10)</f>
         <v>44.85</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H10" s="23">
         <v>187.2</v>
       </c>
-      <c r="I10" s="39">
+      <c r="I10" s="23">
         <v>594.88</v>
       </c>
     </row>
@@ -2427,26 +2427,26 @@
       <c r="B11" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="39">
+      <c r="C11" s="23">
         <v>0.6</v>
       </c>
-      <c r="D11" s="39">
+      <c r="D11" s="23">
         <v>1.2</v>
       </c>
-      <c r="E11" s="39">
+      <c r="E11" s="23">
         <v>2.1</v>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="23">
         <v>3</v>
       </c>
-      <c r="G11" s="39">
+      <c r="G11" s="23">
         <f>SUM(C11:F11)</f>
         <v>6.9</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H11" s="23">
         <v>32.4</v>
       </c>
-      <c r="I11" s="39">
+      <c r="I11" s="23">
         <v>112.32</v>
       </c>
     </row>
@@ -2454,81 +2454,81 @@
       <c r="B12" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="C12" s="40">
+      <c r="C12" s="24">
         <f>C10+C11</f>
         <v>4.5</v>
       </c>
-      <c r="D12" s="40">
+      <c r="D12" s="24">
         <f>D10+D11</f>
         <v>9</v>
       </c>
-      <c r="E12" s="40">
+      <c r="E12" s="24">
         <f>E10+E11</f>
         <v>15.75</v>
       </c>
-      <c r="F12" s="40">
+      <c r="F12" s="24">
         <f>F10+F11</f>
         <v>22.5</v>
       </c>
-      <c r="G12" s="40">
+      <c r="G12" s="24">
         <f>SUM(G10:G11)</f>
         <v>51.75</v>
       </c>
-      <c r="H12" s="40">
+      <c r="H12" s="24">
         <f>H10+H11</f>
         <v>219.6</v>
       </c>
-      <c r="I12" s="40">
+      <c r="I12" s="24">
         <f>I10+I11</f>
         <v>707.2</v>
       </c>
     </row>
     <row r="13" spans="2:9">
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
     </row>
     <row r="14" spans="2:9">
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="2:9">
       <c r="B15" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C15" s="39">
+      <c r="C15" s="23">
         <v>0.24</v>
       </c>
-      <c r="D15" s="39">
+      <c r="D15" s="23">
         <v>0.48</v>
       </c>
-      <c r="E15" s="39">
+      <c r="E15" s="23">
         <v>0.84</v>
       </c>
-      <c r="F15" s="39">
+      <c r="F15" s="23">
         <v>1.2</v>
       </c>
-      <c r="G15" s="39">
+      <c r="G15" s="23">
         <f>SUM(C15:F15)</f>
         <v>2.76</v>
       </c>
-      <c r="H15" s="39">
+      <c r="H15" s="23">
         <v>12.96</v>
       </c>
-      <c r="I15" s="39">
+      <c r="I15" s="23">
         <v>41.6</v>
       </c>
     </row>
@@ -2536,26 +2536,26 @@
       <c r="B16" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="C16" s="39">
+      <c r="C16" s="23">
         <v>0.3</v>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="23">
         <v>0.6</v>
       </c>
-      <c r="E16" s="39">
+      <c r="E16" s="23">
         <v>1.05</v>
       </c>
-      <c r="F16" s="39">
+      <c r="F16" s="23">
         <v>1.5</v>
       </c>
-      <c r="G16" s="39">
+      <c r="G16" s="23">
         <f>SUM(C16:F16)</f>
         <v>3.45</v>
       </c>
-      <c r="H16" s="39">
+      <c r="H16" s="23">
         <v>16.2</v>
       </c>
-      <c r="I16" s="39">
+      <c r="I16" s="23">
         <v>52</v>
       </c>
     </row>
@@ -2563,26 +2563,26 @@
       <c r="B17" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="39">
+      <c r="C17" s="23">
         <v>0.48</v>
       </c>
-      <c r="D17" s="39">
+      <c r="D17" s="23">
         <v>0.96</v>
       </c>
-      <c r="E17" s="39">
+      <c r="E17" s="23">
         <v>1.68</v>
       </c>
-      <c r="F17" s="39">
+      <c r="F17" s="23">
         <v>2.4</v>
       </c>
-      <c r="G17" s="39">
+      <c r="G17" s="23">
         <f>SUM(C17:F17)</f>
         <v>5.52</v>
       </c>
-      <c r="H17" s="39">
+      <c r="H17" s="23">
         <v>25.92</v>
       </c>
-      <c r="I17" s="39">
+      <c r="I17" s="23">
         <v>83.2</v>
       </c>
     </row>
@@ -2590,26 +2590,26 @@
       <c r="B18" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="C18" s="39">
+      <c r="C18" s="23">
         <v>0.54</v>
       </c>
-      <c r="D18" s="39">
+      <c r="D18" s="23">
         <v>1.08</v>
       </c>
-      <c r="E18" s="39">
+      <c r="E18" s="23">
         <v>1.89</v>
       </c>
-      <c r="F18" s="39">
+      <c r="F18" s="23">
         <v>2.7</v>
       </c>
-      <c r="G18" s="39">
+      <c r="G18" s="23">
         <f>SUM(C18:F18)</f>
         <v>6.21</v>
       </c>
-      <c r="H18" s="39">
+      <c r="H18" s="23">
         <v>23.33</v>
       </c>
-      <c r="I18" s="39">
+      <c r="I18" s="23">
         <v>67.39</v>
       </c>
     </row>
@@ -2617,31 +2617,31 @@
       <c r="B19" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="C19" s="40">
+      <c r="C19" s="24">
         <f t="shared" ref="C19:I19" si="0">SUM(C15:C18)</f>
         <v>1.56</v>
       </c>
-      <c r="D19" s="40">
+      <c r="D19" s="24">
         <f t="shared" si="0"/>
         <v>3.12</v>
       </c>
-      <c r="E19" s="40">
+      <c r="E19" s="24">
         <f t="shared" si="0"/>
         <v>5.46</v>
       </c>
-      <c r="F19" s="40">
+      <c r="F19" s="24">
         <f t="shared" si="0"/>
         <v>7.8</v>
       </c>
-      <c r="G19" s="40">
+      <c r="G19" s="24">
         <f t="shared" si="0"/>
         <v>17.940000000000001</v>
       </c>
-      <c r="H19" s="40">
+      <c r="H19" s="24">
         <f t="shared" si="0"/>
         <v>78.41</v>
       </c>
-      <c r="I19" s="40">
+      <c r="I19" s="24">
         <f t="shared" si="0"/>
         <v>244.19</v>
       </c>
@@ -2650,31 +2650,31 @@
       <c r="B20" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="C20" s="40">
+      <c r="C20" s="24">
         <f t="shared" ref="C20:I20" si="1">C12-C19</f>
         <v>2.94</v>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="24">
         <f t="shared" si="1"/>
         <v>5.88</v>
       </c>
-      <c r="E20" s="40">
+      <c r="E20" s="24">
         <f t="shared" si="1"/>
         <v>10.29</v>
       </c>
-      <c r="F20" s="40">
+      <c r="F20" s="24">
         <f t="shared" si="1"/>
         <v>14.7</v>
       </c>
-      <c r="G20" s="40">
+      <c r="G20" s="24">
         <f t="shared" si="1"/>
         <v>33.81</v>
       </c>
-      <c r="H20" s="40">
+      <c r="H20" s="24">
         <f t="shared" si="1"/>
         <v>141.19</v>
       </c>
-      <c r="I20" s="40">
+      <c r="I20" s="24">
         <f t="shared" si="1"/>
         <v>463.01000000000005</v>
       </c>
@@ -2683,81 +2683,81 @@
       <c r="B21" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C21" s="41">
+      <c r="C21" s="25">
         <f t="shared" ref="C21:I21" si="2">C20/C12</f>
         <v>0.65333333333333332</v>
       </c>
-      <c r="D21" s="41">
+      <c r="D21" s="25">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="E21" s="41">
+      <c r="E21" s="25">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="F21" s="41">
+      <c r="F21" s="25">
         <f t="shared" si="2"/>
         <v>0.65333333333333332</v>
       </c>
-      <c r="G21" s="41">
+      <c r="G21" s="25">
         <f t="shared" si="2"/>
         <v>0.65333333333333343</v>
       </c>
-      <c r="H21" s="41">
+      <c r="H21" s="25">
         <f t="shared" si="2"/>
         <v>0.64294171220400731</v>
       </c>
-      <c r="I21" s="41">
+      <c r="I21" s="25">
         <f t="shared" si="2"/>
         <v>0.65470871040723988</v>
       </c>
     </row>
     <row r="22" spans="2:9">
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
     </row>
     <row r="23" spans="2:9">
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C24" s="39">
+      <c r="C24" s="23">
         <v>3</v>
       </c>
-      <c r="D24" s="39">
+      <c r="D24" s="23">
         <v>3</v>
       </c>
-      <c r="E24" s="39">
+      <c r="E24" s="23">
         <v>4.5</v>
       </c>
-      <c r="F24" s="39">
+      <c r="F24" s="23">
         <v>4.5</v>
       </c>
-      <c r="G24" s="39">
+      <c r="G24" s="23">
         <f>SUM(C24:F24)</f>
         <v>15</v>
       </c>
-      <c r="H24" s="39">
+      <c r="H24" s="23">
         <v>39</v>
       </c>
-      <c r="I24" s="39">
+      <c r="I24" s="23">
         <v>102</v>
       </c>
     </row>
@@ -2765,26 +2765,26 @@
       <c r="B25" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="39">
+      <c r="C25" s="23">
         <v>6</v>
       </c>
-      <c r="D25" s="39">
+      <c r="D25" s="23">
         <v>6</v>
       </c>
-      <c r="E25" s="39">
+      <c r="E25" s="23">
         <v>7.5</v>
       </c>
-      <c r="F25" s="39">
+      <c r="F25" s="23">
         <v>7.5</v>
       </c>
-      <c r="G25" s="39">
+      <c r="G25" s="23">
         <f>SUM(C25:F25)</f>
         <v>27</v>
       </c>
-      <c r="H25" s="39">
+      <c r="H25" s="23">
         <v>42</v>
       </c>
-      <c r="I25" s="39">
+      <c r="I25" s="23">
         <v>78</v>
       </c>
     </row>
@@ -2792,26 +2792,26 @@
       <c r="B26" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="C26" s="39">
+      <c r="C26" s="23">
         <v>1.5</v>
       </c>
-      <c r="D26" s="39">
+      <c r="D26" s="23">
         <v>1.5</v>
       </c>
-      <c r="E26" s="39">
+      <c r="E26" s="23">
         <v>2</v>
       </c>
-      <c r="F26" s="39">
+      <c r="F26" s="23">
         <v>2</v>
       </c>
-      <c r="G26" s="39">
+      <c r="G26" s="23">
         <f>SUM(C26:F26)</f>
         <v>7</v>
       </c>
-      <c r="H26" s="39">
+      <c r="H26" s="23">
         <v>12</v>
       </c>
-      <c r="I26" s="39">
+      <c r="I26" s="23">
         <v>24</v>
       </c>
     </row>
@@ -2819,74 +2819,74 @@
       <c r="B27" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="C27" s="40">
+      <c r="C27" s="24">
         <f t="shared" ref="C27:I27" si="3">SUM(C24:C26)</f>
         <v>10.5</v>
       </c>
-      <c r="D27" s="40">
+      <c r="D27" s="24">
         <f t="shared" si="3"/>
         <v>10.5</v>
       </c>
-      <c r="E27" s="40">
+      <c r="E27" s="24">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="F27" s="40">
+      <c r="F27" s="24">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="G27" s="40">
+      <c r="G27" s="24">
         <f t="shared" si="3"/>
         <v>49</v>
       </c>
-      <c r="H27" s="40">
+      <c r="H27" s="24">
         <f t="shared" si="3"/>
         <v>93</v>
       </c>
-      <c r="I27" s="40">
+      <c r="I27" s="24">
         <f t="shared" si="3"/>
         <v>204</v>
       </c>
     </row>
     <row r="28" spans="2:9">
-      <c r="B28" s="36"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="41"/>
+      <c r="I28" s="41"/>
     </row>
     <row r="29" spans="2:9">
       <c r="B29" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="C29" s="42">
+      <c r="C29" s="26">
         <f t="shared" ref="C29:I29" si="4">C20-C27</f>
         <v>-7.5600000000000005</v>
       </c>
-      <c r="D29" s="42">
+      <c r="D29" s="26">
         <f t="shared" si="4"/>
         <v>-4.62</v>
       </c>
-      <c r="E29" s="42">
+      <c r="E29" s="26">
         <f t="shared" si="4"/>
         <v>-3.7100000000000009</v>
       </c>
-      <c r="F29" s="42">
+      <c r="F29" s="26">
         <f t="shared" si="4"/>
         <v>0.69999999999999929</v>
       </c>
-      <c r="G29" s="42">
+      <c r="G29" s="26">
         <f t="shared" si="4"/>
         <v>-15.189999999999998</v>
       </c>
-      <c r="H29" s="42">
+      <c r="H29" s="26">
         <f t="shared" si="4"/>
         <v>48.19</v>
       </c>
-      <c r="I29" s="42">
+      <c r="I29" s="26">
         <f t="shared" si="4"/>
         <v>259.01000000000005</v>
       </c>
@@ -2895,31 +2895,31 @@
       <c r="B30" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C30" s="41">
+      <c r="C30" s="25">
         <f t="shared" ref="C30:I30" si="5">C29/C12</f>
         <v>-1.6800000000000002</v>
       </c>
-      <c r="D30" s="41">
+      <c r="D30" s="25">
         <f t="shared" si="5"/>
         <v>-0.51333333333333331</v>
       </c>
-      <c r="E30" s="41">
+      <c r="E30" s="25">
         <f t="shared" si="5"/>
         <v>-0.2355555555555556</v>
       </c>
-      <c r="F30" s="41">
+      <c r="F30" s="25">
         <f t="shared" si="5"/>
         <v>3.1111111111111079E-2</v>
       </c>
-      <c r="G30" s="41">
+      <c r="G30" s="25">
         <f t="shared" si="5"/>
         <v>-0.29352657004830912</v>
       </c>
-      <c r="H30" s="41">
+      <c r="H30" s="25">
         <f t="shared" si="5"/>
         <v>0.21944444444444444</v>
       </c>
-      <c r="I30" s="41">
+      <c r="I30" s="25">
         <f t="shared" si="5"/>
         <v>0.36624717194570139</v>
       </c>
@@ -2973,15 +2973,15 @@
       <c r="H3" s="18"/>
     </row>
     <row r="5" spans="2:8">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="42" t="s">
         <v>176</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="14" t="s">
@@ -3156,15 +3156,15 @@
       <c r="H13" s="18"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="43" t="s">
         <v>184</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
     </row>
     <row r="17" spans="2:8">
       <c r="B17" s="14" t="s">

</xml_diff>